<commit_message>
Añadidos pines de controlador ftdi
</commit_message>
<xml_diff>
--- a/00-Documents/05-Generated/Basys3_mt9v111_pins.xlsx
+++ b/00-Documents/05-Generated/Basys3_mt9v111_pins.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cmgomezj\Documents\PERSONAL\WORKSPACE\VICON\00-Documents\05-Generated\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA47B470-C4C3-4432-B0FB-AC3D4654CE8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A8A0DBD-0766-4DBE-9F25-BB41D32A2463}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-18135" yWindow="-120" windowWidth="18240" windowHeight="28320" xr2:uid="{15C29769-F0EB-4CAA-8B36-813084D4AB6B}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{15C29769-F0EB-4CAA-8B36-813084D4AB6B}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
+    <sheet name="Hoja2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="120">
   <si>
     <t>ZYBO Z7 PMOD</t>
   </si>
@@ -297,16 +298,121 @@
   </si>
   <si>
     <t>PMOD PIN3</t>
+  </si>
+  <si>
+    <t>D0</t>
+  </si>
+  <si>
+    <t>D1</t>
+  </si>
+  <si>
+    <t>D2</t>
+  </si>
+  <si>
+    <t>D3</t>
+  </si>
+  <si>
+    <t>D4</t>
+  </si>
+  <si>
+    <t>D5</t>
+  </si>
+  <si>
+    <t>D6</t>
+  </si>
+  <si>
+    <t>D7</t>
+  </si>
+  <si>
+    <t>C1</t>
+  </si>
+  <si>
+    <t>C2</t>
+  </si>
+  <si>
+    <t>C3</t>
+  </si>
+  <si>
+    <t>C4</t>
+  </si>
+  <si>
+    <t>C5</t>
+  </si>
+  <si>
+    <t>C6</t>
+  </si>
+  <si>
+    <t>C7</t>
+  </si>
+  <si>
+    <t>JB</t>
+  </si>
+  <si>
+    <t>C0</t>
+  </si>
+  <si>
+    <t>A14</t>
+  </si>
+  <si>
+    <t>A15</t>
+  </si>
+  <si>
+    <t>A16</t>
+  </si>
+  <si>
+    <t>A17</t>
+  </si>
+  <si>
+    <t>B15</t>
+  </si>
+  <si>
+    <t>C15</t>
+  </si>
+  <si>
+    <t>B16</t>
+  </si>
+  <si>
+    <t>C16</t>
+  </si>
+  <si>
+    <t>K17</t>
+  </si>
+  <si>
+    <t>L17</t>
+  </si>
+  <si>
+    <t>M18</t>
+  </si>
+  <si>
+    <t>M19</t>
+  </si>
+  <si>
+    <t>N17</t>
+  </si>
+  <si>
+    <t>P17</t>
+  </si>
+  <si>
+    <t>P18</t>
+  </si>
+  <si>
+    <t>R18</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -347,7 +453,25 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="10">
+  <dxfs count="16">
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -392,21 +516,34 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{FB4DB42A-B270-49D9-8E7E-B57EA1782BC1}" name="Tabla1" displayName="Tabla1" ref="A1:I25" totalsRowShown="0" headerRowDxfId="0" dataDxfId="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{FB4DB42A-B270-49D9-8E7E-B57EA1782BC1}" name="Tabla1" displayName="Tabla1" ref="A1:I25" totalsRowShown="0" headerRowDxfId="15" dataDxfId="14">
   <autoFilter ref="A1:I25" xr:uid="{FB4DB42A-B270-49D9-8E7E-B57EA1782BC1}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:I25">
     <sortCondition ref="A1:A25"/>
   </sortState>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{913992E7-7039-4CBE-A28B-B5EEECEA5F8F}" name="SIGNAL" dataDxfId="9"/>
-    <tableColumn id="3" xr3:uid="{AB712527-EF50-42E3-B1E6-EE92D386FCF9}" name="ZYBO Z7 PMOD" dataDxfId="8"/>
-    <tableColumn id="4" xr3:uid="{5D76D5AA-8822-439F-870D-94D2FD684EAA}" name="PMOD PIN" dataDxfId="7"/>
-    <tableColumn id="5" xr3:uid="{67953FC4-43AD-4AAC-838A-89D103EBF702}" name="FPGA PIN" dataDxfId="6"/>
-    <tableColumn id="7" xr3:uid="{95D35D42-61B6-4F67-88AF-3B1E6EF4FB6D}" name="BASYS 3 PMOD" dataDxfId="5"/>
-    <tableColumn id="8" xr3:uid="{839B4710-6E2F-438F-A337-A12D7DADBE8B}" name="PMOD PIN3" dataDxfId="4"/>
-    <tableColumn id="9" xr3:uid="{E387078C-5520-4C3A-BE0F-59042D4D8EC8}" name="FPGA PIN2" dataDxfId="3"/>
+    <tableColumn id="1" xr3:uid="{913992E7-7039-4CBE-A28B-B5EEECEA5F8F}" name="SIGNAL" dataDxfId="13"/>
+    <tableColumn id="3" xr3:uid="{AB712527-EF50-42E3-B1E6-EE92D386FCF9}" name="ZYBO Z7 PMOD" dataDxfId="12"/>
+    <tableColumn id="4" xr3:uid="{5D76D5AA-8822-439F-870D-94D2FD684EAA}" name="PMOD PIN" dataDxfId="11"/>
+    <tableColumn id="5" xr3:uid="{67953FC4-43AD-4AAC-838A-89D103EBF702}" name="FPGA PIN" dataDxfId="10"/>
+    <tableColumn id="7" xr3:uid="{95D35D42-61B6-4F67-88AF-3B1E6EF4FB6D}" name="BASYS 3 PMOD" dataDxfId="9"/>
+    <tableColumn id="8" xr3:uid="{839B4710-6E2F-438F-A337-A12D7DADBE8B}" name="PMOD PIN3" dataDxfId="8"/>
+    <tableColumn id="9" xr3:uid="{E387078C-5520-4C3A-BE0F-59042D4D8EC8}" name="FPGA PIN2" dataDxfId="7"/>
     <tableColumn id="10" xr3:uid="{D2F489F0-0532-42C5-A393-2255C06A746E}" name="MT9V111 Description"/>
-    <tableColumn id="11" xr3:uid="{A2612E40-9605-4A11-B6F9-373299C9C575}" name="MT9V111 Type" dataDxfId="2"/>
+    <tableColumn id="11" xr3:uid="{A2612E40-9605-4A11-B6F9-373299C9C575}" name="MT9V111 Type" dataDxfId="6"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{EDD32A04-E3D4-45B9-8502-A7CEF02BE9CF}" name="Tabla2" displayName="Tabla2" ref="A1:D17" totalsRowShown="0" headerRowDxfId="1" dataDxfId="0">
+  <autoFilter ref="A1:D17" xr:uid="{EDD32A04-E3D4-45B9-8502-A7CEF02BE9CF}"/>
+  <tableColumns count="4">
+    <tableColumn id="1" xr3:uid="{4351CA45-F1F2-4B15-AEE7-704967498C48}" name="SIGNAL" dataDxfId="5"/>
+    <tableColumn id="2" xr3:uid="{E44582F1-386B-43A3-A3A6-FA4D0FFDB6B3}" name="BASYS 3 PMOD" dataDxfId="4"/>
+    <tableColumn id="3" xr3:uid="{AEC0817C-3E9F-4018-847F-94E33A10BBF1}" name="PMOD PIN" dataDxfId="3"/>
+    <tableColumn id="4" xr3:uid="{FF53CFA7-3F7D-4623-AE44-48D2B8F43634}" name="FPGA PIN" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -735,10 +872,10 @@
     <col min="1" max="1" width="11.42578125" style="1" customWidth="1"/>
     <col min="2" max="2" width="16.28515625" style="1" customWidth="1"/>
     <col min="3" max="3" width="12.28515625" style="1" customWidth="1"/>
-    <col min="4" max="4" width="11.42578125" style="1"/>
+    <col min="4" max="4" width="13.85546875" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="16.28515625" style="1" customWidth="1"/>
     <col min="6" max="6" width="13.28515625" style="1" customWidth="1"/>
-    <col min="7" max="7" width="12.42578125" style="1" customWidth="1"/>
+    <col min="7" max="7" width="14.85546875" style="1" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="46.140625" style="2" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="15.5703125" style="1" customWidth="1"/>
     <col min="10" max="16384" width="11.42578125" style="1"/>
@@ -1451,4 +1588,264 @@
     <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{55863B70-3A6E-4AC3-A500-01006B6154F2}">
+  <dimension ref="A1:D17"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="11.42578125" style="1"/>
+    <col min="2" max="2" width="16.28515625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="12.28515625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="11.42578125" style="1"/>
+    <col min="5" max="5" width="19.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="16384" width="11.42578125" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="C2" s="1">
+        <v>1</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="C3" s="1">
+        <v>7</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="C4" s="1">
+        <v>2</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="C5" s="1">
+        <v>8</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="C6" s="1">
+        <v>3</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="C7" s="1">
+        <v>9</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="C8" s="1">
+        <v>4</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="C9" s="1">
+        <v>10</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C10" s="1">
+        <v>1</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C11" s="1">
+        <v>7</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C12" s="1">
+        <v>2</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C13" s="1">
+        <v>8</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C14" s="1">
+        <v>3</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C15" s="1">
+        <v>9</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C16" s="1">
+        <v>4</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C17" s="1">
+        <v>10</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>119</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>